<commit_message>
HH farm: N via HH_FARM_N/argv; log batch of 3 applies
Allow small scheduled batches without editing the script. Refresh Excel report after Swordfish, RWB/Wildberries Bank, and DigiKey responses.

Co-authored-by: marmot-smr <marmot-smr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/resume/hh-otkliki-30.xlsx
+++ b/resume/hh-otkliki-30.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,52 +471,48 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LLC Лоция</t>
+          <t>Swordfish Security</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Системный аналитик</t>
+          <t>Системный аналитик (AppSec.Wave)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>офис</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://hh.ru/vacancy/136886384</t>
+          <t>https://hh.ru/vacancy/138778279</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>застрял на опроснике</t>
+          <t>отклик (уже подтверждён после клика)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>застрял на опроснике</t>
+          <t>простой отклик (клик)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>Здравствуйте!
-Откликаюсь на роль Системный аналитик в LLC Лоция. Сейчас System Analyst Middle+ в Ви6 Сервисес: интеграции с WMS и государственными ИС, БТ/ФТ/ТЗ, постановки с критериями приёмки.
-Близко к вакансии по стеку: Swagger, SQL, REST. Описываю REST в OpenAPI, сценарии Kafka/RabbitMQ, SQL к PostgreSQL, UML и BPMN. Кейс: трудозатраты процесса снизились в два раза по торговой сети.
+Откликаюсь на роль Системный аналитик в Swordfish Security. Сейчас System Analyst Middle+ в Ви6 Сервисес: интеграции с WMS и государственными ИС, БТ/ФТ/ТЗ, постановки с критериями приёмки.
+Близко к вакансии по стеку: SQL, REST, BPMN. Описываю REST в OpenAPI, сценарии Kafka/RabbitMQ, SQL к PostgreSQL, UML и BPMN. Кейс: трудозатраты процесса снизились в два раза по торговой сети.
 Английский C1. Москва, гибрид или удалённо. Готов обсудить задачи на этой неделе.
 Telegram: surkov_danila</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-22T20:22:23.250061+00:00</t>
+          <t>2026-10-23T09:10:02.872052+00:00</t>
         </is>
       </c>
     </row>
@@ -528,19 +524,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LLC Антара</t>
+          <t>RWB (Wildberries &amp; Russ)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Системный аналитик (банковский сектор)</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>up to 230 000 ₽ per month, after taxes</t>
-        </is>
-      </c>
+          <t>Системный аналитик в Wildberries Bank</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>офис</t>
@@ -548,7 +540,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://hh.ru/vacancy/138137648</t>
+          <t>https://hh.ru/vacancy/138636682</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -564,167 +556,67 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>Здравствуйте!
-Откликаюсь на роль Системный аналитик в LLC Антара. Сейчас System Analyst Middle+ в Ви6 Сервисес: интеграции с WMS и государственными ИС, БТ/ФТ/ТЗ, постановки с критериями приёмки.
-Близко к вакансии по стеку: SQL, REST, BPMN. Описываю REST в OpenAPI, сценарии Kafka/RabbitMQ, SQL к PostgreSQL, UML и BPMN. Кейс: трудозатраты процесса снизились в два раза по торговой сети.
+Откликаюсь на роль Системный аналитик в Wildberries Bank в RWB (Wildberries &amp; Russ). Сейчас System Analyst Middle+ в Ви6 Сервисес: интеграции с WMS и государственными ИС, БТ/ФТ/ТЗ, постановки с критериями приёмки.
+Близко к вакансии по стеку: SQL, BPMN, UML. Описываю REST в OpenAPI, сценарии Kafka/RabbitMQ, SQL к PostgreSQL, UML и BPMN. Кейс: трудозатраты процесса снизились в два раза по торговой сети.
 Английский C1. Москва, гибрид или удалённо. Готов обсудить задачи на этой неделе.
 Telegram: surkov_danila</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-22T20:22:56.590541+00:00</t>
+          <t>2026-10-23T09:10:37.967884+00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bell Integrator</t>
+          <t>DigiKey Limited</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Системный аналитик (Мобильная разработка)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>офис</t>
-        </is>
-      </c>
+          <t>Системный аналитик</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>from 150 000 up to 220 000 ₽ per month, after taxes</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://hh.ru/vacancy/137673521</t>
+          <t>https://hh.ru/vacancy/138624964</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>застрял на опроснике</t>
+          <t>отклик+письмо+опрос</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>застрял на опроснике</t>
+          <t>отклик + сопроводительное</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>Здравствуйте!
-Откликаюсь на роль Системный аналитик в Bell Integrator. Сейчас System Analyst Middle+ в Ви6 Сервисес: интеграции с WMS и государственными ИС, БТ/ФТ/ТЗ, постановки с критериями приёмки.
-Близко к вакансии по стеку: OpenAPI, Swagger, PostgreSQL. Описываю REST в OpenAPI, сценарии Kafka/RabbitMQ, SQL к PostgreSQL, UML и BPMN. Кейс: трудозатраты процесса снизились в два раза по торговой сети.
+Откликаюсь на роль Системный аналитик в DigiKey Limited. Сейчас System Analyst Middle+ в Ви6 Сервисес: интеграции с WMS и государственными ИС, БТ/ФТ/ТЗ, постановки с критериями приёмки.
+Близко к вакансии по стеку: OpenAPI, Swagger, SQL. Описываю REST в OpenAPI, сценарии Kafka/RabbitMQ, SQL к PostgreSQL, UML и BPMN. Кейс: трудозатраты процесса снизились в два раза по торговой сети.
 Английский C1. Москва, гибрид или удалённо. Готов обсудить задачи на этой неделе.
 Telegram: surkov_danila</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-22T20:23:25.625180+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Бизнес Автоматизатор</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Системный аналитик / CRM-интегратор (AmoCRM и Битрикс24)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>from 60 000 up to 100 000 ₽ per month, after taxes</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://hh.ru/vacancy/138493514</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>отклик (уже подтверждён после клика)</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>простой отклик (клик)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Здравствуйте!
-Откликаюсь на роль Системный аналитик / CRM-интегратор в Бизнес Автоматизатор. Сейчас System Analyst Middle+ в Ви6 Сервисес: интеграции с WMS и государственными ИС, БТ/ФТ/ТЗ, постановки с критериями приёмки.
-Близко к вакансии по стеку: REST, BPMN, интеграции. Описываю REST в OpenAPI, сценарии Kafka/RabbitMQ, SQL к PostgreSQL, UML и BPMN. Кейс: трудозатраты процесса снизились в два раза по торговой сети.
-Английский C1. Москва, гибрид или удалённо. Готов обсудить задачи на этой неделе.
-Telegram: surkov_danila</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2026-10-22T20:24:02.606318+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>LLC АЙФЭЛЛ</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Системный аналитик</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://hh.ru/vacancy/137673406</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>отклик (уже подтверждён после клика)</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>простой отклик (клик)</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Здравствуйте!
-Откликаюсь на роль Системный аналитик в LLC АЙФЭЛЛ. Сейчас System Analyst Middle+ в Ви6 Сервисес: интеграции с WMS и государственными ИС, БТ/ФТ/ТЗ, постановки с критериями приёмки.
-Близко к вакансии по стеку: Swagger, Kafka, RabbitMQ. Описываю REST в OpenAPI, сценарии Kafka/RabbitMQ, SQL к PostgreSQL, UML и BPMN. Кейс: трудозатраты процесса снизились в два раза по торговой сети.
-Английский C1. Москва, гибрид или удалённо. Готов обсудить задачи на этой неделе.
-Telegram: surkov_danila</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2026-10-22T20:24:41.794362+00:00</t>
+          <t>2026-10-23T09:11:14.666782+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>